<commit_message>
persona + ujm + usability
</commit_message>
<xml_diff>
--- a/P1/Usability-review.xlsx
+++ b/P1/Usability-review.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documentos Importantes\IN INF\4º\DIU\DIU1.JMDA\P1\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="870" yWindow="885" windowWidth="3975" windowHeight="3765"/>
+    <workbookView xWindow="876" yWindow="888" windowWidth="3972" windowHeight="3768"/>
   </bookViews>
   <sheets>
     <sheet name="Valoración Usabilidad" sheetId="1" r:id="rId1"/>
@@ -12,8 +17,7 @@
     <sheet name="Usability guidelines" sheetId="3" r:id="rId3"/>
     <sheet name="Rating ranges" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="145621"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataSignature="AMtx7mi6SXC1K0cfcIj2UxcE1drm7aHxgQ=="/>
@@ -28,7 +32,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="J1" authorId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -51,7 +55,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="B9" authorId="0">
+    <comment ref="B9" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -67,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B11" authorId="0">
+    <comment ref="B11" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -83,7 +87,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B13" authorId="0">
+    <comment ref="B13" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -99,7 +103,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B15" authorId="0">
+    <comment ref="B15" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -115,7 +119,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B17" authorId="0">
+    <comment ref="B17" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -131,7 +135,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B21" authorId="0">
+    <comment ref="B21" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -147,7 +151,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B23" authorId="0">
+    <comment ref="B23" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -163,7 +167,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B25" authorId="0">
+    <comment ref="B25" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -179,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B29" authorId="0">
+    <comment ref="B29" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -195,7 +199,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B31" authorId="0">
+    <comment ref="B31" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -211,7 +215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B33" authorId="0">
+    <comment ref="B33" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -227,7 +231,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B35" authorId="0">
+    <comment ref="B35" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -243,7 +247,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B37" authorId="0">
+    <comment ref="B37" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -259,7 +263,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B39" authorId="0">
+    <comment ref="B39" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -275,7 +279,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B41" authorId="0">
+    <comment ref="B41" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -291,7 +295,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B43" authorId="0">
+    <comment ref="B43" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -307,7 +311,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B45" authorId="0">
+    <comment ref="B45" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -323,7 +327,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B49" authorId="0">
+    <comment ref="B49" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -339,7 +343,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B51" authorId="0">
+    <comment ref="B51" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -355,7 +359,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B53" authorId="0">
+    <comment ref="B53" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -371,7 +375,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B55" authorId="0">
+    <comment ref="B55" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -387,7 +391,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B59" authorId="0">
+    <comment ref="B59" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -403,7 +407,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B61" authorId="0">
+    <comment ref="B61" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -419,7 +423,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B63" authorId="0">
+    <comment ref="B63" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -435,7 +439,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B67" authorId="0">
+    <comment ref="B67" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -451,7 +455,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B69" authorId="0">
+    <comment ref="B69" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -467,7 +471,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B71" authorId="0">
+    <comment ref="B71" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -483,7 +487,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B73" authorId="0">
+    <comment ref="B73" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -499,7 +503,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B75" authorId="0">
+    <comment ref="B75" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -515,7 +519,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B79" authorId="0">
+    <comment ref="B79" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -531,7 +535,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B81" authorId="0">
+    <comment ref="B81" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -547,7 +551,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B83" authorId="0">
+    <comment ref="B83" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -563,7 +567,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B85" authorId="0">
+    <comment ref="B85" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -579,7 +583,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B89" authorId="0">
+    <comment ref="B89" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -595,7 +599,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B91" authorId="0">
+    <comment ref="B91" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -611,7 +615,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B93" authorId="0">
+    <comment ref="B93" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -627,7 +631,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B95" authorId="0">
+    <comment ref="B95" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -643,7 +647,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B97" authorId="0">
+    <comment ref="B97" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -659,7 +663,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B101" authorId="0">
+    <comment ref="B101" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -675,7 +679,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B103" authorId="0">
+    <comment ref="B103" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -691,7 +695,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B105" authorId="0">
+    <comment ref="B105" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -707,7 +711,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B107" authorId="0">
+    <comment ref="B107" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -723,7 +727,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B111" authorId="0">
+    <comment ref="B111" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -739,7 +743,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B113" authorId="0">
+    <comment ref="B113" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -755,7 +759,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B115" authorId="0">
+    <comment ref="B115" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -781,7 +785,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="226">
   <si>
     <t>Usability guidelines</t>
   </si>
@@ -1853,11 +1857,71 @@
   <si>
     <t>Ramen Shifu</t>
   </si>
+  <si>
+    <t>Unicamente te pide tu nombre, email y taberna habitual.</t>
+  </si>
+  <si>
+    <t>Los campos requeridos están marcados con un asterisco. No hay campos opcionales.</t>
+  </si>
+  <si>
+    <t>Hay un menú desplegable para seleccionar tu taberna.</t>
+  </si>
+  <si>
+    <t>El formulario para inscribirse a la newsletter es muy sencillo, no tiene pasos ni indicador de progreso.</t>
+  </si>
+  <si>
+    <t>No se proporcionan ejemplos ni se especifica formato. Por la sencillez del formulario no supone un problema grave.</t>
+  </si>
+  <si>
+    <t>El error aparece debaajo del campo afectado. Los mensajes son genericos.</t>
+  </si>
+  <si>
+    <t>Misma justificación, mensajes genericos.</t>
+  </si>
+  <si>
+    <t>El error aparece una vez intentas enviar el formulario, no en tiempo real.</t>
+  </si>
+  <si>
+    <t>Al producirse un error, el formulario mantiene todos los datos introducidos.</t>
+  </si>
+  <si>
+    <t>La carta está bien explicada. Cada item tiene una imagen y una descripción con los ingredientes.</t>
+  </si>
+  <si>
+    <t>La seccion del blog contiene numerosos enlaces, por ejemplo de colaboraciones. Los iconos de redes sociales también son puntos de salida.</t>
+  </si>
+  <si>
+    <t>El contenido está bien escrito y los platos del menú bien definidos. Los ingredientes japoneses podrían estár mejor explicados, pero se puede argumentar que no es un problema de cara al publico objetivo de este restaurante.</t>
+  </si>
+  <si>
+    <t>La terminología es consistente en toda la web (nombres de platos, de locales, menús…)</t>
+  </si>
+  <si>
+    <t>La letra es de tamaño adecuado y tipografía facil de leer. Los fondos de colores pastel ayudan a contrastar el texto y que sea más facil de leer.</t>
+  </si>
+  <si>
+    <t>En la web no se realizan operaciones complejas que requieran de menús de ayuda contextual.</t>
+  </si>
+  <si>
+    <t>Mismo razonamiento.</t>
+  </si>
+  <si>
+    <t>Cada local tiene su numero de telefono facilmente visible en la cabecera de la subpagina correspondiente.</t>
+  </si>
+  <si>
+    <t>Si desde la pagina principal pulsas el boton "Carta" que se encuentra en la cabecera te dirige a una pagina protegida por contraseña. Este error no sucede al acceder a la carta de una localización concreta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La web carga razonablemente rápido, incluidas las imagenes. </t>
+  </si>
+  <si>
+    <t>Admite distintos navegadores. El formulario en movil parece no reconocer bien la resolucion de la pantalla.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -2474,13 +2538,16 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2498,16 +2565,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2542,6 +2606,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2812,35 +2879,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" customWidth="1"/>
-    <col min="2" max="2" width="60.28515625" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="4.42578125" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="4.140625" customWidth="1"/>
-    <col min="9" max="9" width="51.28515625" customWidth="1"/>
-    <col min="10" max="10" width="2.140625" customWidth="1"/>
-    <col min="11" max="12" width="12.140625" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" customWidth="1"/>
+    <col min="2" max="2" width="60.33203125" customWidth="1"/>
+    <col min="3" max="3" width="4.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="4.44140625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="4.109375" customWidth="1"/>
+    <col min="9" max="9" width="51.33203125" customWidth="1"/>
+    <col min="10" max="10" width="2.109375" customWidth="1"/>
+    <col min="11" max="12" width="12.109375" customWidth="1"/>
+    <col min="13" max="13" width="9.109375" customWidth="1"/>
     <col min="14" max="26" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="23.25" customHeight="1">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="86" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="98"/>
-      <c r="I1" s="99"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="88"/>
       <c r="J1" s="4"/>
       <c r="K1" s="6"/>
       <c r="L1" s="5"/>
@@ -2887,10 +2954,10 @@
       <c r="V2" s="10"/>
     </row>
     <row r="3" spans="1:22" ht="24" customHeight="1">
-      <c r="A3" s="100" t="s">
+      <c r="A3" s="89" t="s">
         <v>205</v>
       </c>
-      <c r="B3" s="86"/>
+      <c r="B3" s="90"/>
       <c r="C3" s="23"/>
       <c r="D3" s="24" t="s">
         <v>10</v>
@@ -3017,19 +3084,19 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
-      <c r="K7" s="85" t="s">
+      <c r="K7" s="100" t="s">
         <v>30</v>
       </c>
-      <c r="L7" s="85" t="s">
+      <c r="L7" s="100" t="s">
         <v>31</v>
       </c>
-      <c r="M7" s="85" t="s">
+      <c r="M7" s="100" t="s">
         <v>32</v>
       </c>
-      <c r="N7" s="87" t="s">
+      <c r="N7" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="O7" s="87" t="s">
+      <c r="O7" s="101" t="s">
         <v>33</v>
       </c>
       <c r="P7" s="18"/>
@@ -3054,11 +3121,11 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
-      <c r="K8" s="86"/>
-      <c r="L8" s="86"/>
-      <c r="M8" s="86"/>
-      <c r="N8" s="86"/>
-      <c r="O8" s="86"/>
+      <c r="K8" s="90"/>
+      <c r="L8" s="90"/>
+      <c r="M8" s="90"/>
+      <c r="N8" s="90"/>
+      <c r="O8" s="90"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="39"/>
@@ -3829,7 +3896,7 @@
         <f>A31+1</f>
         <v>11</v>
       </c>
-      <c r="B33" s="102" t="s">
+      <c r="B33" s="85" t="s">
         <v>101</v>
       </c>
       <c r="C33" s="1"/>
@@ -4012,7 +4079,7 @@
         <f>A37+1</f>
         <v>14</v>
       </c>
-      <c r="B39" s="102" t="s">
+      <c r="B39" s="85" t="s">
         <v>107</v>
       </c>
       <c r="C39" s="1"/>
@@ -4208,7 +4275,7 @@
         <f>A43+1</f>
         <v>17</v>
       </c>
-      <c r="B45" s="102" t="s">
+      <c r="B45" s="85" t="s">
         <v>113</v>
       </c>
       <c r="C45" s="1"/>
@@ -4302,7 +4369,7 @@
         <f>A45+1</f>
         <v>18</v>
       </c>
-      <c r="B49" s="102" t="s">
+      <c r="B49" s="85" t="s">
         <v>115</v>
       </c>
       <c r="C49" s="1"/>
@@ -4814,7 +4881,7 @@
       </c>
       <c r="C67" s="1"/>
       <c r="D67" s="43" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E67" s="1"/>
       <c r="F67" s="1" t="e">
@@ -4826,7 +4893,9 @@
         <v>#REF!</v>
       </c>
       <c r="H67" s="1"/>
-      <c r="I67" s="44"/>
+      <c r="I67" s="44" t="s">
+        <v>209</v>
+      </c>
       <c r="J67" s="1"/>
       <c r="K67" s="45">
         <v>3</v>
@@ -4837,15 +4906,15 @@
       </c>
       <c r="M67" s="47">
         <f>VLOOKUP(D67,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N67" s="47">
         <f>M67*L67</f>
-        <v>0</v>
+        <v>1.7999999999999998</v>
       </c>
       <c r="O67" s="47">
         <f>IF(M67=0,0,L67*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68" spans="1:15" ht="12" customHeight="1">
@@ -4875,7 +4944,7 @@
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="43" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E69" s="1"/>
       <c r="F69" s="1" t="e">
@@ -4887,7 +4956,9 @@
         <v>#REF!</v>
       </c>
       <c r="H69" s="1"/>
-      <c r="I69" s="44"/>
+      <c r="I69" s="44" t="s">
+        <v>206</v>
+      </c>
       <c r="J69" s="1"/>
       <c r="K69" s="45">
         <v>2</v>
@@ -4898,15 +4969,15 @@
       </c>
       <c r="M69" s="47">
         <f>VLOOKUP(D69,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N69" s="47">
         <f>M69*L69</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="O69" s="47">
         <f>IF(M69=0,0,L69*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:15" ht="12" customHeight="1">
@@ -4936,7 +5007,7 @@
       </c>
       <c r="C71" s="1"/>
       <c r="D71" s="43" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E71" s="1"/>
       <c r="F71" s="1" t="e">
@@ -4948,7 +5019,9 @@
         <v>#REF!</v>
       </c>
       <c r="H71" s="1"/>
-      <c r="I71" s="44"/>
+      <c r="I71" s="44" t="s">
+        <v>207</v>
+      </c>
       <c r="J71" s="1"/>
       <c r="K71" s="45">
         <v>2</v>
@@ -4959,15 +5032,15 @@
       </c>
       <c r="M71" s="47">
         <f>VLOOKUP(D71,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N71" s="47">
         <f>M71*L71</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O71" s="47">
         <f>IF(M71=0,0,L71*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:15" ht="12" customHeight="1">
@@ -4997,7 +5070,7 @@
       </c>
       <c r="C73" s="1"/>
       <c r="D73" s="43" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E73" s="1"/>
       <c r="F73" s="1" t="e">
@@ -5009,7 +5082,9 @@
         <v>#REF!</v>
       </c>
       <c r="H73" s="1"/>
-      <c r="I73" s="44"/>
+      <c r="I73" s="44" t="s">
+        <v>208</v>
+      </c>
       <c r="J73" s="1"/>
       <c r="K73" s="45">
         <v>3</v>
@@ -5020,15 +5095,15 @@
       </c>
       <c r="M73" s="47">
         <f>VLOOKUP(D73,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N73" s="47">
         <f>M73*L73</f>
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="O73" s="47">
         <f>IF(M73=0,0,L73*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74" spans="1:15" ht="12" customHeight="1">
@@ -5058,7 +5133,7 @@
       </c>
       <c r="C75" s="1"/>
       <c r="D75" s="43" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E75" s="1"/>
       <c r="F75" s="1" t="e">
@@ -5070,7 +5145,9 @@
         <v>#REF!</v>
       </c>
       <c r="H75" s="1"/>
-      <c r="I75" s="44"/>
+      <c r="I75" s="44" t="s">
+        <v>210</v>
+      </c>
       <c r="J75" s="1"/>
       <c r="K75" s="45">
         <v>3</v>
@@ -5081,15 +5158,15 @@
       </c>
       <c r="M75" s="47">
         <f>VLOOKUP(D75,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N75" s="47">
         <f>M75*L75</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="O75" s="47">
         <f>IF(M75=0,0,L75*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76" spans="1:15" ht="12" customHeight="1">
@@ -5152,7 +5229,7 @@
       </c>
       <c r="C79" s="1"/>
       <c r="D79" s="43" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E79" s="1"/>
       <c r="F79" s="1" t="e">
@@ -5164,7 +5241,9 @@
         <v>#REF!</v>
       </c>
       <c r="H79" s="1"/>
-      <c r="I79" s="44"/>
+      <c r="I79" s="44" t="s">
+        <v>211</v>
+      </c>
       <c r="J79" s="1"/>
       <c r="K79" s="45">
         <v>4</v>
@@ -5175,15 +5254,15 @@
       </c>
       <c r="M79" s="47">
         <f>VLOOKUP(D79,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N79" s="47">
         <f>M79*L79</f>
-        <v>0</v>
+        <v>2.4000000000000004</v>
       </c>
       <c r="O79" s="47">
         <f>IF(M79=0,0,L79*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="80" spans="1:15" ht="12" customHeight="1">
@@ -5213,7 +5292,7 @@
       </c>
       <c r="C81" s="1"/>
       <c r="D81" s="43" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E81" s="1"/>
       <c r="F81" s="1" t="e">
@@ -5225,7 +5304,9 @@
         <v>#REF!</v>
       </c>
       <c r="H81" s="1"/>
-      <c r="I81" s="44"/>
+      <c r="I81" s="44" t="s">
+        <v>212</v>
+      </c>
       <c r="J81" s="1"/>
       <c r="K81" s="45">
         <v>3</v>
@@ -5236,15 +5317,15 @@
       </c>
       <c r="M81" s="47">
         <f>VLOOKUP(D81,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N81" s="47">
         <f>M81*L81</f>
-        <v>0</v>
+        <v>1.7999999999999998</v>
       </c>
       <c r="O81" s="47">
         <f>IF(M81=0,0,L81*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82" spans="1:15" ht="12" customHeight="1">
@@ -5274,7 +5355,7 @@
       </c>
       <c r="C83" s="1"/>
       <c r="D83" s="43" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E83" s="1"/>
       <c r="F83" s="1" t="e">
@@ -5286,7 +5367,9 @@
         <v>#REF!</v>
       </c>
       <c r="H83" s="1"/>
-      <c r="I83" s="44"/>
+      <c r="I83" s="44" t="s">
+        <v>213</v>
+      </c>
       <c r="J83" s="1"/>
       <c r="K83" s="45">
         <v>3</v>
@@ -5297,15 +5380,15 @@
       </c>
       <c r="M83" s="47">
         <f>VLOOKUP(D83,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N83" s="47">
         <f>M83*L83</f>
-        <v>0</v>
+        <v>1.7999999999999998</v>
       </c>
       <c r="O83" s="47">
         <f>IF(M83=0,0,L83*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84" spans="1:15" ht="12" customHeight="1">
@@ -5335,7 +5418,7 @@
       </c>
       <c r="C85" s="1"/>
       <c r="D85" s="43" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E85" s="1"/>
       <c r="F85" s="1" t="e">
@@ -5347,7 +5430,9 @@
         <v>#REF!</v>
       </c>
       <c r="H85" s="1"/>
-      <c r="I85" s="44"/>
+      <c r="I85" s="44" t="s">
+        <v>214</v>
+      </c>
       <c r="J85" s="1"/>
       <c r="K85" s="45">
         <v>3</v>
@@ -5358,15 +5443,15 @@
       </c>
       <c r="M85" s="47">
         <f>VLOOKUP(D85,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N85" s="47">
         <f>M85*L85</f>
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="O85" s="47">
         <f>IF(M85=0,0,L85*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86" spans="1:15" ht="12" customHeight="1">
@@ -5429,7 +5514,7 @@
       </c>
       <c r="C89" s="1"/>
       <c r="D89" s="43" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E89" s="1"/>
       <c r="F89" s="1" t="e">
@@ -5441,7 +5526,9 @@
         <v>#REF!</v>
       </c>
       <c r="H89" s="1"/>
-      <c r="I89" s="44"/>
+      <c r="I89" s="44" t="s">
+        <v>215</v>
+      </c>
       <c r="J89" s="1"/>
       <c r="K89" s="45">
         <v>5</v>
@@ -5452,15 +5539,15 @@
       </c>
       <c r="M89" s="47">
         <f>VLOOKUP(D89,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N89" s="47">
         <f>M89*L89</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O89" s="47">
         <f>IF(M89=0,0,L89*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90" spans="1:15" ht="12" customHeight="1">
@@ -5490,7 +5577,7 @@
       </c>
       <c r="C91" s="1"/>
       <c r="D91" s="43" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E91" s="1"/>
       <c r="F91" s="1" t="e">
@@ -5502,7 +5589,9 @@
         <v>#REF!</v>
       </c>
       <c r="H91" s="1"/>
-      <c r="I91" s="44"/>
+      <c r="I91" s="44" t="s">
+        <v>216</v>
+      </c>
       <c r="J91" s="1"/>
       <c r="K91" s="45">
         <v>2</v>
@@ -5513,15 +5602,15 @@
       </c>
       <c r="M91" s="47">
         <f>VLOOKUP(D91,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N91" s="47">
         <f>M91*L91</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="O91" s="47">
         <f>IF(M91=0,0,L91*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92" spans="1:15" ht="12" customHeight="1">
@@ -5551,7 +5640,7 @@
       </c>
       <c r="C93" s="1"/>
       <c r="D93" s="43" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E93" s="1"/>
       <c r="F93" s="1" t="e">
@@ -5563,7 +5652,9 @@
         <v>#REF!</v>
       </c>
       <c r="H93" s="1"/>
-      <c r="I93" s="44"/>
+      <c r="I93" s="44" t="s">
+        <v>217</v>
+      </c>
       <c r="J93" s="1"/>
       <c r="K93" s="45">
         <v>4</v>
@@ -5574,15 +5665,15 @@
       </c>
       <c r="M93" s="47">
         <f>VLOOKUP(D93,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N93" s="47">
         <f>M93*L93</f>
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="O93" s="47">
         <f>IF(M93=0,0,L93*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94" spans="1:15" ht="12" customHeight="1">
@@ -5612,7 +5703,7 @@
       </c>
       <c r="C95" s="1"/>
       <c r="D95" s="43" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E95" s="1"/>
       <c r="F95" s="1" t="e">
@@ -5624,7 +5715,9 @@
         <v>#REF!</v>
       </c>
       <c r="H95" s="1"/>
-      <c r="I95" s="44"/>
+      <c r="I95" s="44" t="s">
+        <v>218</v>
+      </c>
       <c r="J95" s="1"/>
       <c r="K95" s="45">
         <v>3</v>
@@ -5635,15 +5728,15 @@
       </c>
       <c r="M95" s="47">
         <f>VLOOKUP(D95,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N95" s="47">
         <f>M95*L95</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O95" s="47">
         <f>IF(M95=0,0,L95*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="96" spans="1:15" ht="12" customHeight="1">
@@ -5673,7 +5766,7 @@
       </c>
       <c r="C97" s="1"/>
       <c r="D97" s="43" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E97" s="1"/>
       <c r="F97" s="1" t="e">
@@ -5685,7 +5778,9 @@
         <v>#REF!</v>
       </c>
       <c r="H97" s="1"/>
-      <c r="I97" s="44"/>
+      <c r="I97" s="44" t="s">
+        <v>219</v>
+      </c>
       <c r="J97" s="1"/>
       <c r="K97" s="45">
         <v>3</v>
@@ -5696,15 +5791,15 @@
       </c>
       <c r="M97" s="47">
         <f>VLOOKUP(D97,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N97" s="47">
         <f>M97*L97</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O97" s="47">
         <f>IF(M97=0,0,L97*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="98" spans="1:26" ht="12" customHeight="1">
@@ -5767,7 +5862,7 @@
       </c>
       <c r="C101" s="1"/>
       <c r="D101" s="43" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="E101" s="1"/>
       <c r="F101" s="1" t="e">
@@ -5779,7 +5874,9 @@
         <v>#REF!</v>
       </c>
       <c r="H101" s="1"/>
-      <c r="I101" s="44"/>
+      <c r="I101" s="44" t="s">
+        <v>220</v>
+      </c>
       <c r="J101" s="1"/>
       <c r="K101" s="45">
         <v>4</v>
@@ -5828,7 +5925,7 @@
       </c>
       <c r="C103" s="1"/>
       <c r="D103" s="43" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="E103" s="1"/>
       <c r="F103" s="1" t="e">
@@ -5840,7 +5937,9 @@
         <v>#REF!</v>
       </c>
       <c r="H103" s="1"/>
-      <c r="I103" s="44"/>
+      <c r="I103" s="44" t="s">
+        <v>221</v>
+      </c>
       <c r="J103" s="1"/>
       <c r="K103" s="45">
         <v>3</v>
@@ -5889,7 +5988,7 @@
       </c>
       <c r="C105" s="1"/>
       <c r="D105" s="43" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="E105" s="1"/>
       <c r="F105" s="1" t="e">
@@ -5901,7 +6000,9 @@
         <v>#REF!</v>
       </c>
       <c r="H105" s="1"/>
-      <c r="I105" s="44"/>
+      <c r="I105" s="44" t="s">
+        <v>221</v>
+      </c>
       <c r="J105" s="1"/>
       <c r="K105" s="45">
         <v>3</v>
@@ -5950,7 +6051,7 @@
       </c>
       <c r="C107" s="1"/>
       <c r="D107" s="43" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E107" s="1"/>
       <c r="F107" s="1" t="e">
@@ -5962,7 +6063,9 @@
         <v>#REF!</v>
       </c>
       <c r="H107" s="1"/>
-      <c r="I107" s="44"/>
+      <c r="I107" s="44" t="s">
+        <v>222</v>
+      </c>
       <c r="J107" s="1"/>
       <c r="K107" s="45">
         <v>2</v>
@@ -5973,15 +6076,15 @@
       </c>
       <c r="M107" s="47">
         <f>VLOOKUP(D107,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N107" s="47">
         <f>M107*L107</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="O107" s="47">
         <f>IF(M107=0,0,L107*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:26" ht="12" customHeight="1">
@@ -6044,7 +6147,7 @@
       </c>
       <c r="C111" s="13"/>
       <c r="D111" s="43" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="E111" s="13"/>
       <c r="F111" s="13" t="e">
@@ -6056,7 +6159,9 @@
         <v>#REF!</v>
       </c>
       <c r="H111" s="13"/>
-      <c r="I111" s="44"/>
+      <c r="I111" s="44" t="s">
+        <v>224</v>
+      </c>
       <c r="J111" s="13"/>
       <c r="K111" s="34">
         <v>4</v>
@@ -6067,15 +6172,15 @@
       </c>
       <c r="M111" s="66">
         <f>VLOOKUP(D111,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N111" s="66">
         <f>M111*L111</f>
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="O111" s="66">
         <f>IF(M111=0,0,L111*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P111" s="13"/>
       <c r="Q111" s="13"/>
@@ -6127,7 +6232,7 @@
       </c>
       <c r="C113" s="13"/>
       <c r="D113" s="71" t="s">
-        <v>4</v>
+        <v>146</v>
       </c>
       <c r="E113" s="13"/>
       <c r="F113" s="13" t="e">
@@ -6139,7 +6244,9 @@
         <v>#REF!</v>
       </c>
       <c r="H113" s="13"/>
-      <c r="I113" s="44"/>
+      <c r="I113" s="44" t="s">
+        <v>223</v>
+      </c>
       <c r="J113" s="13"/>
       <c r="K113" s="34">
         <v>4</v>
@@ -6150,15 +6257,15 @@
       </c>
       <c r="M113" s="66">
         <f>VLOOKUP(D113,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N113" s="66">
         <f>M113*L113</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="O113" s="66">
         <f>IF(M113=0,0,L113*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P113" s="13"/>
       <c r="Q113" s="13"/>
@@ -6210,7 +6317,7 @@
       </c>
       <c r="C115" s="13"/>
       <c r="D115" s="43" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E115" s="13"/>
       <c r="F115" s="13" t="e">
@@ -6222,7 +6329,9 @@
         <v>#REF!</v>
       </c>
       <c r="H115" s="13"/>
-      <c r="I115" s="44"/>
+      <c r="I115" s="44" t="s">
+        <v>225</v>
+      </c>
       <c r="J115" s="13"/>
       <c r="K115" s="34">
         <v>3</v>
@@ -6233,15 +6342,15 @@
       </c>
       <c r="M115" s="66">
         <f>VLOOKUP(D115,Q1:R9,2,FALSE)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N115" s="66">
         <f>M115*L115</f>
-        <v>0</v>
+        <v>1.7999999999999998</v>
       </c>
       <c r="O115" s="66">
         <f>IF(M115=0,0,L115*MAX(R2:R8))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P115" s="13"/>
       <c r="Q115" s="13"/>
@@ -6279,7 +6388,7 @@
       <c r="C117" s="73"/>
       <c r="D117" s="74">
         <f>IF(ISERR((N117/O117)*100),"",(N117/O117)*100)</f>
-        <v>92</v>
+        <v>82.162162162162161</v>
       </c>
       <c r="E117" s="75"/>
       <c r="F117" s="75"/>
@@ -6290,11 +6399,11 @@
       </c>
       <c r="I117" s="77" t="str">
         <f>VLOOKUP(J117,'Rating ranges'!A2:B7,2,TRUE)</f>
-        <v>Excellent</v>
+        <v>Good</v>
       </c>
       <c r="J117" s="7">
         <f>IF(D117="",0,D117)</f>
-        <v>92</v>
+        <v>82.162162162162161</v>
       </c>
       <c r="K117" s="68">
         <f>MAX(K9:K115)</f>
@@ -6304,11 +6413,11 @@
       <c r="M117" s="68"/>
       <c r="N117" s="69">
         <f t="shared" ref="N117:O117" si="0">SUM(N9:N115)</f>
-        <v>50.599999999999994</v>
+        <v>91.199999999999989</v>
       </c>
       <c r="O117" s="69">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>111</v>
       </c>
     </row>
     <row r="118" spans="1:26" ht="13.5" customHeight="1">
@@ -6324,90 +6433,90 @@
       <c r="M118" s="1"/>
     </row>
     <row r="119" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A119" s="88" t="str">
+      <c r="A119" s="91" t="str">
         <f>"* Very poor (less than "&amp;('Rating ranges'!A4)&amp;") - Users are likely to experience very significant difficulties using this site or system and might not be able to complete a significant number of important tasks."</f>
         <v>* Very poor (less than 29) - Users are likely to experience very significant difficulties using this site or system and might not be able to complete a significant number of important tasks.</v>
       </c>
-      <c r="B119" s="89"/>
-      <c r="C119" s="89"/>
-      <c r="D119" s="89"/>
-      <c r="E119" s="89"/>
-      <c r="F119" s="89"/>
-      <c r="G119" s="89"/>
-      <c r="H119" s="89"/>
-      <c r="I119" s="90"/>
+      <c r="B119" s="92"/>
+      <c r="C119" s="92"/>
+      <c r="D119" s="92"/>
+      <c r="E119" s="92"/>
+      <c r="F119" s="92"/>
+      <c r="G119" s="92"/>
+      <c r="H119" s="92"/>
+      <c r="I119" s="93"/>
       <c r="J119" s="1"/>
       <c r="K119" s="16"/>
       <c r="L119" s="16"/>
       <c r="M119" s="1"/>
     </row>
     <row r="120" spans="1:26" ht="15" customHeight="1">
-      <c r="A120" s="91" t="str">
+      <c r="A120" s="94" t="str">
         <f>"* Poor (between "&amp;('Rating ranges'!A4)&amp;" and "&amp;('Rating ranges'!A5)&amp;") - Users are likely to experience some difficulties using this site or system and might not be able to complete some important tasks."</f>
         <v>* Poor (between 29 and 49) - Users are likely to experience some difficulties using this site or system and might not be able to complete some important tasks.</v>
       </c>
-      <c r="B120" s="86"/>
-      <c r="C120" s="86"/>
-      <c r="D120" s="86"/>
-      <c r="E120" s="86"/>
-      <c r="F120" s="86"/>
-      <c r="G120" s="86"/>
-      <c r="H120" s="86"/>
-      <c r="I120" s="92"/>
+      <c r="B120" s="90"/>
+      <c r="C120" s="90"/>
+      <c r="D120" s="90"/>
+      <c r="E120" s="90"/>
+      <c r="F120" s="90"/>
+      <c r="G120" s="90"/>
+      <c r="H120" s="90"/>
+      <c r="I120" s="95"/>
       <c r="J120" s="1"/>
       <c r="K120" s="16"/>
       <c r="L120" s="16"/>
       <c r="M120" s="1"/>
     </row>
     <row r="121" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A121" s="93" t="str">
+      <c r="A121" s="96" t="str">
         <f>"* Moderate (between "&amp;('Rating ranges'!A5)&amp;" and "&amp;('Rating ranges'!A6)&amp;") - Users should be able to use this site or system and complete most important tasks, however the user experience could be significantly improved."</f>
         <v>* Moderate (between 49 and 69) - Users should be able to use this site or system and complete most important tasks, however the user experience could be significantly improved.</v>
       </c>
-      <c r="B121" s="86"/>
-      <c r="C121" s="86"/>
-      <c r="D121" s="86"/>
-      <c r="E121" s="86"/>
-      <c r="F121" s="86"/>
-      <c r="G121" s="86"/>
-      <c r="H121" s="86"/>
-      <c r="I121" s="92"/>
+      <c r="B121" s="90"/>
+      <c r="C121" s="90"/>
+      <c r="D121" s="90"/>
+      <c r="E121" s="90"/>
+      <c r="F121" s="90"/>
+      <c r="G121" s="90"/>
+      <c r="H121" s="90"/>
+      <c r="I121" s="95"/>
       <c r="J121" s="1"/>
       <c r="K121" s="16"/>
       <c r="L121" s="16"/>
       <c r="M121" s="1"/>
     </row>
     <row r="122" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A122" s="91" t="str">
+      <c r="A122" s="94" t="str">
         <f>"* Good (between "&amp;('Rating ranges'!A6)&amp;" and "&amp;('Rating ranges'!A7)&amp;") - Users should be able to use this site or system with relative ease and should be able to complete the vast majority of important tasks."</f>
         <v>* Good (between 69 and 89) - Users should be able to use this site or system with relative ease and should be able to complete the vast majority of important tasks.</v>
       </c>
-      <c r="B122" s="86"/>
-      <c r="C122" s="86"/>
-      <c r="D122" s="86"/>
-      <c r="E122" s="86"/>
-      <c r="F122" s="86"/>
-      <c r="G122" s="86"/>
-      <c r="H122" s="86"/>
-      <c r="I122" s="92"/>
+      <c r="B122" s="90"/>
+      <c r="C122" s="90"/>
+      <c r="D122" s="90"/>
+      <c r="E122" s="90"/>
+      <c r="F122" s="90"/>
+      <c r="G122" s="90"/>
+      <c r="H122" s="90"/>
+      <c r="I122" s="95"/>
       <c r="J122" s="1"/>
       <c r="K122" s="16"/>
       <c r="L122" s="16"/>
       <c r="M122" s="1"/>
     </row>
     <row r="123" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A123" s="94" t="str">
+      <c r="A123" s="97" t="str">
         <f>"* Excellent (more than "&amp;('Rating ranges'!A7)&amp;") - This site or system provides an excellent user experience for users. Users should be able to complete all important tasks on the site or system."</f>
         <v>* Excellent (more than 89) - This site or system provides an excellent user experience for users. Users should be able to complete all important tasks on the site or system.</v>
       </c>
-      <c r="B123" s="95"/>
-      <c r="C123" s="95"/>
-      <c r="D123" s="95"/>
-      <c r="E123" s="95"/>
-      <c r="F123" s="95"/>
-      <c r="G123" s="95"/>
-      <c r="H123" s="95"/>
-      <c r="I123" s="96"/>
+      <c r="B123" s="98"/>
+      <c r="C123" s="98"/>
+      <c r="D123" s="98"/>
+      <c r="E123" s="98"/>
+      <c r="F123" s="98"/>
+      <c r="G123" s="98"/>
+      <c r="H123" s="98"/>
+      <c r="I123" s="99"/>
       <c r="J123" s="1"/>
       <c r="K123" s="16"/>
       <c r="L123" s="16"/>
@@ -16950,18 +17059,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="A122:I122"/>
+    <mergeCell ref="A123:I123"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="M7:M8"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A119:I119"/>
     <mergeCell ref="A120:I120"/>
     <mergeCell ref="A121:I121"/>
-    <mergeCell ref="A122:I122"/>
-    <mergeCell ref="A123:I123"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
   </mergeCells>
   <conditionalFormatting sqref="D111 D113 D115 D105 D107 D101 D103 D89 D91 D93 D95 D97 D79 D81 D83 D85 D69 D71 D73 D75 D67 D63 D59 D61 D49 D51 D53 D55 D29 D35 D37 D39 D41 D43 D45 D31:D33 D21 D23:D25 D17 D9 D11 D13 D15">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
@@ -16993,35 +17102,35 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" customWidth="1"/>
-    <col min="2" max="2" width="60.28515625" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="4.42578125" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="4.140625" customWidth="1"/>
-    <col min="9" max="9" width="51.28515625" customWidth="1"/>
-    <col min="10" max="10" width="2.140625" customWidth="1"/>
-    <col min="11" max="12" width="12.140625" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" customWidth="1"/>
+    <col min="2" max="2" width="60.33203125" customWidth="1"/>
+    <col min="3" max="3" width="4.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="4.44140625" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="4.109375" customWidth="1"/>
+    <col min="9" max="9" width="51.33203125" customWidth="1"/>
+    <col min="10" max="10" width="2.109375" customWidth="1"/>
+    <col min="11" max="12" width="12.109375" customWidth="1"/>
+    <col min="13" max="13" width="9.109375" customWidth="1"/>
     <col min="14" max="26" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="23.25" customHeight="1">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="98"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="98"/>
-      <c r="I1" s="99"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="88"/>
       <c r="J1" s="1"/>
       <c r="K1" s="3"/>
       <c r="L1" s="5"/>
@@ -17068,10 +17177,10 @@
       <c r="V2" s="10"/>
     </row>
     <row r="3" spans="1:22" ht="24" customHeight="1">
-      <c r="A3" s="100" t="s">
+      <c r="A3" s="89" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="86"/>
+      <c r="B3" s="90"/>
       <c r="C3" s="23"/>
       <c r="D3" s="24" t="s">
         <v>10</v>
@@ -17198,19 +17307,19 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
-      <c r="K7" s="85" t="s">
+      <c r="K7" s="100" t="s">
         <v>30</v>
       </c>
-      <c r="L7" s="85" t="s">
+      <c r="L7" s="100" t="s">
         <v>31</v>
       </c>
-      <c r="M7" s="85" t="s">
+      <c r="M7" s="100" t="s">
         <v>32</v>
       </c>
-      <c r="N7" s="87" t="s">
+      <c r="N7" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="O7" s="87" t="s">
+      <c r="O7" s="101" t="s">
         <v>33</v>
       </c>
       <c r="P7" s="18"/>
@@ -17235,11 +17344,11 @@
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
-      <c r="K8" s="86"/>
-      <c r="L8" s="86"/>
-      <c r="M8" s="86"/>
-      <c r="N8" s="86"/>
-      <c r="O8" s="86"/>
+      <c r="K8" s="90"/>
+      <c r="L8" s="90"/>
+      <c r="M8" s="90"/>
+      <c r="N8" s="90"/>
+      <c r="O8" s="90"/>
       <c r="P8" s="18"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="39"/>
@@ -20459,90 +20568,90 @@
       <c r="M118" s="1"/>
     </row>
     <row r="119" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A119" s="88" t="str">
+      <c r="A119" s="91" t="str">
         <f>"* Very poor (less than "&amp;('Rating ranges'!A4)&amp;") - Users are likely to experience very significant difficulties using this site or system and might not be able to complete a significant number of important tasks."</f>
         <v>* Very poor (less than 29) - Users are likely to experience very significant difficulties using this site or system and might not be able to complete a significant number of important tasks.</v>
       </c>
-      <c r="B119" s="89"/>
-      <c r="C119" s="89"/>
-      <c r="D119" s="89"/>
-      <c r="E119" s="89"/>
-      <c r="F119" s="89"/>
-      <c r="G119" s="89"/>
-      <c r="H119" s="89"/>
-      <c r="I119" s="90"/>
+      <c r="B119" s="92"/>
+      <c r="C119" s="92"/>
+      <c r="D119" s="92"/>
+      <c r="E119" s="92"/>
+      <c r="F119" s="92"/>
+      <c r="G119" s="92"/>
+      <c r="H119" s="92"/>
+      <c r="I119" s="93"/>
       <c r="J119" s="1"/>
       <c r="K119" s="16"/>
       <c r="L119" s="16"/>
       <c r="M119" s="1"/>
     </row>
     <row r="120" spans="1:26" ht="15" customHeight="1">
-      <c r="A120" s="91" t="str">
+      <c r="A120" s="94" t="str">
         <f>"* Poor (between "&amp;('Rating ranges'!A4)&amp;" and "&amp;('Rating ranges'!A5)&amp;") - Users are likely to experience some difficulties using this site or system and might not be able to complete some important tasks."</f>
         <v>* Poor (between 29 and 49) - Users are likely to experience some difficulties using this site or system and might not be able to complete some important tasks.</v>
       </c>
-      <c r="B120" s="86"/>
-      <c r="C120" s="86"/>
-      <c r="D120" s="86"/>
-      <c r="E120" s="86"/>
-      <c r="F120" s="86"/>
-      <c r="G120" s="86"/>
-      <c r="H120" s="86"/>
-      <c r="I120" s="92"/>
+      <c r="B120" s="90"/>
+      <c r="C120" s="90"/>
+      <c r="D120" s="90"/>
+      <c r="E120" s="90"/>
+      <c r="F120" s="90"/>
+      <c r="G120" s="90"/>
+      <c r="H120" s="90"/>
+      <c r="I120" s="95"/>
       <c r="J120" s="1"/>
       <c r="K120" s="16"/>
       <c r="L120" s="16"/>
       <c r="M120" s="1"/>
     </row>
     <row r="121" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A121" s="93" t="str">
+      <c r="A121" s="96" t="str">
         <f>"* Moderate (between "&amp;('Rating ranges'!A5)&amp;" and "&amp;('Rating ranges'!A6)&amp;") - Users should be able to use this site or system and complete most important tasks, however the user experience could be significantly improved."</f>
         <v>* Moderate (between 49 and 69) - Users should be able to use this site or system and complete most important tasks, however the user experience could be significantly improved.</v>
       </c>
-      <c r="B121" s="86"/>
-      <c r="C121" s="86"/>
-      <c r="D121" s="86"/>
-      <c r="E121" s="86"/>
-      <c r="F121" s="86"/>
-      <c r="G121" s="86"/>
-      <c r="H121" s="86"/>
-      <c r="I121" s="92"/>
+      <c r="B121" s="90"/>
+      <c r="C121" s="90"/>
+      <c r="D121" s="90"/>
+      <c r="E121" s="90"/>
+      <c r="F121" s="90"/>
+      <c r="G121" s="90"/>
+      <c r="H121" s="90"/>
+      <c r="I121" s="95"/>
       <c r="J121" s="1"/>
       <c r="K121" s="16"/>
       <c r="L121" s="16"/>
       <c r="M121" s="1"/>
     </row>
     <row r="122" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A122" s="91" t="str">
+      <c r="A122" s="94" t="str">
         <f>"* Good (between "&amp;('Rating ranges'!A6)&amp;" and "&amp;('Rating ranges'!A7)&amp;") - Users should be able to use this site or system with relative ease and should be able to complete the vast majority of important tasks."</f>
         <v>* Good (between 69 and 89) - Users should be able to use this site or system with relative ease and should be able to complete the vast majority of important tasks.</v>
       </c>
-      <c r="B122" s="86"/>
-      <c r="C122" s="86"/>
-      <c r="D122" s="86"/>
-      <c r="E122" s="86"/>
-      <c r="F122" s="86"/>
-      <c r="G122" s="86"/>
-      <c r="H122" s="86"/>
-      <c r="I122" s="92"/>
+      <c r="B122" s="90"/>
+      <c r="C122" s="90"/>
+      <c r="D122" s="90"/>
+      <c r="E122" s="90"/>
+      <c r="F122" s="90"/>
+      <c r="G122" s="90"/>
+      <c r="H122" s="90"/>
+      <c r="I122" s="95"/>
       <c r="J122" s="1"/>
       <c r="K122" s="16"/>
       <c r="L122" s="16"/>
       <c r="M122" s="1"/>
     </row>
     <row r="123" spans="1:26" ht="12.75" customHeight="1">
-      <c r="A123" s="94" t="str">
+      <c r="A123" s="97" t="str">
         <f>"* Excellent (more than "&amp;('Rating ranges'!A7)&amp;") - This site or system provides an excellent user experience for users. Users should be able to complete all important tasks on the site or system."</f>
         <v>* Excellent (more than 89) - This site or system provides an excellent user experience for users. Users should be able to complete all important tasks on the site or system.</v>
       </c>
-      <c r="B123" s="95"/>
-      <c r="C123" s="95"/>
-      <c r="D123" s="95"/>
-      <c r="E123" s="95"/>
-      <c r="F123" s="95"/>
-      <c r="G123" s="95"/>
-      <c r="H123" s="95"/>
-      <c r="I123" s="96"/>
+      <c r="B123" s="98"/>
+      <c r="C123" s="98"/>
+      <c r="D123" s="98"/>
+      <c r="E123" s="98"/>
+      <c r="F123" s="98"/>
+      <c r="G123" s="98"/>
+      <c r="H123" s="98"/>
+      <c r="I123" s="99"/>
       <c r="J123" s="1"/>
       <c r="K123" s="16"/>
       <c r="L123" s="16"/>
@@ -31077,6 +31186,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A119:I119"/>
+    <mergeCell ref="A120:I120"/>
+    <mergeCell ref="A121:I121"/>
+    <mergeCell ref="A122:I122"/>
+    <mergeCell ref="A123:I123"/>
     <mergeCell ref="N7:N8"/>
     <mergeCell ref="O7:O8"/>
     <mergeCell ref="A1:I1"/>
@@ -31084,11 +31198,6 @@
     <mergeCell ref="K7:K8"/>
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="M7:M8"/>
-    <mergeCell ref="A119:I119"/>
-    <mergeCell ref="A120:I120"/>
-    <mergeCell ref="A121:I121"/>
-    <mergeCell ref="A122:I122"/>
-    <mergeCell ref="A123:I123"/>
   </mergeCells>
   <conditionalFormatting sqref="D111 D113 D115 D105 D107 D101 D103 D89 D91 D93 D95 D97 D79 D81 D83 D85 D69 D71 D73 D75 D67 D63 D59 D61 D49 D51 D53 D55 D29 D35 D37 D39 D41 D43 D45 D31:D33 D21 D23:D25 D17 D9 D11 D13 D15">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
@@ -31116,20 +31225,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.140625" customWidth="1"/>
-    <col min="2" max="2" width="103.5703125" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" customWidth="1"/>
+    <col min="2" max="2" width="103.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" customWidth="1"/>
     <col min="4" max="26" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="23.25" customHeight="1">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="98"/>
-      <c r="C1" s="99"/>
+      <c r="B1" s="87"/>
+      <c r="C1" s="88"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1">
       <c r="B2" s="2"/>
@@ -35765,14 +35874,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" customWidth="1"/>
-    <col min="4" max="4" width="5.5703125" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="5.7109375" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" customWidth="1"/>
+    <col min="4" max="4" width="5.5546875" customWidth="1"/>
+    <col min="5" max="5" width="4.6640625" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" customWidth="1"/>
     <col min="7" max="26" width="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -35783,12 +35892,12 @@
       <c r="B1" s="60" t="s">
         <v>144</v>
       </c>
-      <c r="C1" s="101" t="s">
+      <c r="C1" s="102" t="s">
         <v>145</v>
       </c>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
     </row>
     <row r="2" spans="1:6" ht="12.75" customHeight="1">
       <c r="A2" s="61">

</xml_diff>